<commit_message>
Remove temporary Excel file and enhance proforma generation with new cost driver functions
- Deleted temporary Excel file from the repository.
- Added functions in generate_proforma.py to identify the primary cost driver and the first scale trigger based on subscriber levels, improving cost analysis capabilities.
- Updated dashboard and risk reporting to reflect new cost driver calculations.
</commit_message>
<xml_diff>
--- a/docs/DealGapIQ_Financial_Proforma.xlsx
+++ b/docs/DealGapIQ_Financial_Proforma.xlsx
@@ -389,7 +389,7 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Profitability'!$A$8:$A$28</f>
+              <f>'Profitability'!$A$7:$A$28</f>
             </numRef>
           </cat>
           <val>
@@ -502,7 +502,7 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Profitability'!$A$8:$A$28</f>
+              <f>'Profitability'!$A$7:$A$28</f>
             </numRef>
           </cat>
           <val>
@@ -526,7 +526,7 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Profitability'!$A$8:$A$28</f>
+              <f>'Profitability'!$A$7:$A$28</f>
             </numRef>
           </cat>
           <val>
@@ -550,7 +550,7 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Profitability'!$A$8:$A$28</f>
+              <f>'Profitability'!$A$7:$A$28</f>
             </numRef>
           </cat>
           <val>
@@ -574,7 +574,7 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Profitability'!$A$8:$A$28</f>
+              <f>'Profitability'!$A$7:$A$28</f>
             </numRef>
           </cat>
           <val>
@@ -1350,7 +1350,7 @@
     <col width="19" customWidth="1" min="2" max="2"/>
     <col width="24" customWidth="1" min="3" max="3"/>
     <col width="24" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
@@ -1412,7 +1412,7 @@
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>Primary Cost Driver</t>
+          <t>Top Cost @ 100 Subs</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
@@ -1429,12 +1429,12 @@
       </c>
       <c r="C8" s="7" t="inlineStr">
         <is>
-          <t>RentCast (51%)</t>
+          <t>RentCast (46%)</t>
         </is>
       </c>
       <c r="E8" s="7" t="inlineStr">
         <is>
-          <t>~48–80 subs</t>
+          <t>~100 subs (RapidAPI — Redfin)</t>
         </is>
       </c>
     </row>
@@ -8506,7 +8506,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
-    <col width="32" customWidth="1" min="2" max="2"/>
+    <col width="33" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="40" customWidth="1" min="4" max="4"/>
   </cols>
@@ -8556,7 +8556,7 @@
       </c>
       <c r="B5" s="48" t="inlineStr">
         <is>
-          <t>High — 51% of base costs</t>
+          <t>High — 46% of costs @ 100 subs</t>
         </is>
       </c>
       <c r="C5" s="10" t="inlineStr">

</xml_diff>